<commit_message>
novas atualizações e correções e melhorias
novas atualizações e correções e melhorias
</commit_message>
<xml_diff>
--- a/Enviar_email/Cadastro_Fornecedores.xlsx
+++ b/Enviar_email/Cadastro_Fornecedores.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Fabio\Desenvolvimento\Varejo\Enviar_email\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{447A0F22-D880-45AB-B568-F09CD3EDF25D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCF09329-3BA5-4F98-BE24-4C3FF9A486C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="Cadastro_Fornecedores" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Cadastro_Fornecedores">Cadastro_Fornecedores!$B$1:$BO$5</definedName>
+    <definedName name="Cadastro_Fornecedores">Cadastro_Fornecedores!$B$1:$BO$4</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="77">
   <si>
     <t>E-mail 2</t>
   </si>
@@ -244,18 +244,6 @@
     <t>149.810.540.115</t>
   </si>
   <si>
-    <t>XAXIM</t>
-  </si>
-  <si>
-    <t>75818849000176</t>
-  </si>
-  <si>
-    <t>251755770</t>
-  </si>
-  <si>
-    <t>Seca</t>
-  </si>
-  <si>
     <t>novosprojetosbr@gmail.com</t>
   </si>
   <si>
@@ -265,22 +253,7 @@
     <t>fabioacordeiro@yahoo.com.br</t>
   </si>
   <si>
-    <t>fabioacordeiro@hotmail.com; novosprojetosbr@gmail.com</t>
-  </si>
-  <si>
     <t>Email</t>
-  </si>
-  <si>
-    <t>bruno_branco@carrefour.com</t>
-  </si>
-  <si>
-    <t>leonardo_ypiranga@carrefour.com</t>
-  </si>
-  <si>
-    <t>vitor_alves@carrefour.com</t>
-  </si>
-  <si>
-    <t>felipe_santana_6@carrefour.com</t>
   </si>
 </sst>
 </file>
@@ -636,7 +609,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BO9"/>
+  <dimension ref="A1:BO4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="50.88671875" bestFit="1" customWidth="1"/>
@@ -645,7 +618,7 @@
   <sheetData>
     <row r="1" spans="1:67" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="J1" t="s">
         <v>0</v>
@@ -824,7 +797,7 @@
     </row>
     <row r="2" spans="1:67" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="J2" t="s">
         <v>58</v>
@@ -970,7 +943,7 @@
     </row>
     <row r="3" spans="1:67" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="M3" t="b">
         <v>0</v>
@@ -1125,7 +1098,7 @@
     </row>
     <row r="4" spans="1:67" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="J4" t="s">
         <v>65</v>
@@ -1288,181 +1261,6 @@
       </c>
       <c r="BO4" s="1">
         <v>45450.419699074097</v>
-      </c>
-    </row>
-    <row r="5" spans="1:67" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="M5" t="b">
-        <v>1</v>
-      </c>
-      <c r="N5" t="s">
-        <v>67</v>
-      </c>
-      <c r="O5" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>53</v>
-      </c>
-      <c r="S5" t="b">
-        <v>0</v>
-      </c>
-      <c r="U5" t="s">
-        <v>73</v>
-      </c>
-      <c r="W5" t="s">
-        <v>74</v>
-      </c>
-      <c r="X5" t="s">
-        <v>75</v>
-      </c>
-      <c r="Y5" t="s">
-        <v>76</v>
-      </c>
-      <c r="Z5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AA5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AD5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AE5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AF5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AG5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AH5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AI5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AJ5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AL5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AN5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AO5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AP5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AQ5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AR5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AS5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AT5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AU5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AV5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AW5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AX5" t="b">
-        <v>1</v>
-      </c>
-      <c r="AY5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AZ5" t="b">
-        <v>0</v>
-      </c>
-      <c r="BA5" t="b">
-        <v>0</v>
-      </c>
-      <c r="BB5" t="b">
-        <v>0</v>
-      </c>
-      <c r="BC5" t="b">
-        <v>0</v>
-      </c>
-      <c r="BD5" t="b">
-        <v>0</v>
-      </c>
-      <c r="BE5" t="b">
-        <v>0</v>
-      </c>
-      <c r="BF5" t="b">
-        <v>1</v>
-      </c>
-      <c r="BG5" t="b">
-        <v>0</v>
-      </c>
-      <c r="BH5" t="b">
-        <v>0</v>
-      </c>
-      <c r="BI5" t="b">
-        <v>0</v>
-      </c>
-      <c r="BJ5" t="b">
-        <v>0</v>
-      </c>
-      <c r="BK5" t="b">
-        <v>0</v>
-      </c>
-      <c r="BL5" t="b">
-        <v>0</v>
-      </c>
-      <c r="BM5" t="b">
-        <v>0</v>
-      </c>
-      <c r="BN5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:67" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="7" spans="1:67" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="8" spans="1:67" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="9" spans="1:67" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -1470,11 +1268,6 @@
     <hyperlink ref="A3" r:id="rId1" xr:uid="{5520B7B0-BB18-4F2E-BC60-CC658162A40F}"/>
     <hyperlink ref="A2" r:id="rId2" xr:uid="{29B157C2-5962-41BC-879E-7B718B8023AA}"/>
     <hyperlink ref="A4" r:id="rId3" xr:uid="{277CF47B-58C3-49E3-918B-3F086AF8940B}"/>
-    <hyperlink ref="A5" r:id="rId4" display="fabioacordeiro@hotmail.com; " xr:uid="{1AD99D42-069E-4820-BC66-3696553AC940}"/>
-    <hyperlink ref="A6" r:id="rId5" xr:uid="{6A02BEA0-1DFC-41BF-ACD2-DC12E3BCFA70}"/>
-    <hyperlink ref="A7" r:id="rId6" xr:uid="{1E50AB76-50DD-4FF3-BB89-29AE8731AFBC}"/>
-    <hyperlink ref="A8" r:id="rId7" xr:uid="{246DA3B9-FC7F-4AAB-948B-A3885C25E5B8}"/>
-    <hyperlink ref="A9" r:id="rId8" xr:uid="{0685BD1D-16D5-4A84-AE50-0880EC9F9662}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>